<commit_message>
Sistemazione calcolo qtà fattibile interna ed esterna su testata
</commit_message>
<xml_diff>
--- a/Documenti/WorkInProgress.xlsx
+++ b/Documenti/WorkInProgress.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Fattibilit-ODP\Documenti\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://divimast-my.sharepoint.com/personal/mattia_mille_divimast_it/Documents/Desktop/MM/Business Central/Fattibilit-ODP/Documenti/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D59083F2-D5AB-4846-B08E-8FBF6F98D8E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{D59083F2-D5AB-4846-B08E-8FBF6F98D8E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E8E94F9-693C-4FF6-9AD1-15CB5DD1CB33}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="630" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">Verificare fattibilità Z211248 articolo 2308861041	</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>Note</t>
+  </si>
+  <si>
+    <t>Risolto MM 03/02/2026</t>
   </si>
 </sst>
 </file>
@@ -69,12 +72,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -89,10 +98,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -374,14 +384,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="3" width="58.85546875" customWidth="1"/>
-    <col min="4" max="4" width="51.140625" customWidth="1"/>
+    <col min="1" max="2" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="58.88671875" customWidth="1"/>
+    <col min="4" max="4" width="51.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -398,7 +408,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>46055</v>
       </c>
@@ -407,6 +417,9 @@
       </c>
       <c r="C2" t="s">
         <v>0</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Work in progress
</commit_message>
<xml_diff>
--- a/Documenti/WorkInProgress.xlsx
+++ b/Documenti/WorkInProgress.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://divimast-my.sharepoint.com/personal/mattia_mille_divimast_it/Documents/Desktop/MM/Business Central/Fattibilit-ODP/Documenti/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Fattibilit-ODP\Documenti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{D59083F2-D5AB-4846-B08E-8FBF6F98D8E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E8E94F9-693C-4FF6-9AD1-15CB5DD1CB33}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B114CF-E46A-42DC-B3C6-944063E5DF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="630" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
   <si>
     <t xml:space="preserve">Verificare fattibilità Z211248 articolo 2308861041	</t>
   </si>
@@ -49,6 +49,36 @@
   </si>
   <si>
     <t>Risolto MM 03/02/2026</t>
+  </si>
+  <si>
+    <t>AL posto di Terzista --&gt; Area Produzione</t>
+  </si>
+  <si>
+    <t>Escludere Ordini Acq con Ord produzione</t>
+  </si>
+  <si>
+    <t>Aggiugere dopo Expected Tipo numero data 1o elemento</t>
+  </si>
+  <si>
+    <t>Se più di un elemento evidenzare (grassetto?)</t>
+  </si>
+  <si>
+    <t>Aggiungere richiamo monitor avanzamento ovunque c'è in ODP</t>
+  </si>
+  <si>
+    <t>Filtro Tutti solo esterni Solo interni</t>
+  </si>
+  <si>
+    <t>In prima lsta aggiungere codice cliente e nome cliente (ed anche nellultima)</t>
+  </si>
+  <si>
+    <t>Aggiungere filtro Linea produzione e grandezza (flowfield 5406)</t>
+  </si>
+  <si>
+    <t>Evicenziare fattibili in toto da fattibili con trasferimenti</t>
+  </si>
+  <si>
+    <t>Aggiungere campo Exterlan inventory Other Location su 2a lista</t>
   </si>
 </sst>
 </file>
@@ -98,11 +128,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -383,15 +414,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="14.5546875" customWidth="1"/>
-    <col min="3" max="3" width="58.88671875" customWidth="1"/>
-    <col min="4" max="4" width="51.109375" customWidth="1"/>
+    <col min="1" max="2" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="58.85546875" customWidth="1"/>
+    <col min="4" max="4" width="51.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -408,7 +439,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>46055</v>
       </c>
@@ -420,6 +451,116 @@
       </c>
       <c r="D2" s="3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46070</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>